<commit_message>
Update INARA 2026-09-14 12:32:05
</commit_message>
<xml_diff>
--- a/report_cleansing_ps.xlsx
+++ b/report_cleansing_ps.xlsx
@@ -35635,7 +35635,7 @@
         <v>3415</v>
       </c>
       <c r="J844" t="s">
-        <v>3435</v>
+        <v>3436</v>
       </c>
     </row>
     <row r="845" spans="1:10">
@@ -39452,7 +39452,7 @@
         <v>3414</v>
       </c>
       <c r="J969" t="s">
-        <v>3435</v>
+        <v>3436</v>
       </c>
     </row>
     <row r="970" spans="1:10">

</xml_diff>

<commit_message>
Update INARA 2026-09-17 10:50:58
</commit_message>
<xml_diff>
--- a/report_cleansing_ps.xlsx
+++ b/report_cleansing_ps.xlsx
@@ -38924,7 +38924,7 @@
         <v>4959</v>
       </c>
       <c r="J810" t="s">
-        <v>4985</v>
+        <v>4986</v>
       </c>
     </row>
     <row r="811" spans="1:10">
@@ -44852,7 +44852,7 @@
         <v>4982</v>
       </c>
       <c r="J1005" t="s">
-        <v>4985</v>
+        <v>4986</v>
       </c>
     </row>
     <row r="1006" spans="1:10">
@@ -56648,7 +56648,7 @@
         <v>4959</v>
       </c>
       <c r="J1392" t="s">
-        <v>4985</v>
+        <v>4986</v>
       </c>
     </row>
     <row r="1393" spans="1:10">
@@ -60354,7 +60354,7 @@
         <v>4974</v>
       </c>
       <c r="J1514" t="s">
-        <v>4985</v>
+        <v>4986</v>
       </c>
     </row>
     <row r="1515" spans="1:10">
@@ -65518,7 +65518,7 @@
         <v>4966</v>
       </c>
       <c r="J1684" t="s">
-        <v>4985</v>
+        <v>4986</v>
       </c>
     </row>
     <row r="1685" spans="1:10">

</xml_diff>

<commit_message>
Update INARA 2026-09-18 16:34:01
</commit_message>
<xml_diff>
--- a/report_cleansing_ps.xlsx
+++ b/report_cleansing_ps.xlsx
@@ -16782,7 +16782,7 @@
         <v>4955</v>
       </c>
       <c r="J50" t="s">
-        <v>4985</v>
+        <v>4986</v>
       </c>
     </row>
     <row r="51" spans="1:10">
@@ -25830,7 +25830,7 @@
         <v>4951</v>
       </c>
       <c r="J362" t="s">
-        <v>4985</v>
+        <v>4986</v>
       </c>
     </row>
     <row r="363" spans="1:10">
@@ -27367,7 +27367,7 @@
         <v>4951</v>
       </c>
       <c r="J415" t="s">
-        <v>4985</v>
+        <v>4986</v>
       </c>
     </row>
     <row r="416" spans="1:10">
@@ -29394,7 +29394,7 @@
         <v>4951</v>
       </c>
       <c r="J485" t="s">
-        <v>4985</v>
+        <v>4986</v>
       </c>
     </row>
     <row r="486" spans="1:10">
@@ -30293,7 +30293,7 @@
         <v>4951</v>
       </c>
       <c r="J516" t="s">
-        <v>4985</v>
+        <v>4986</v>
       </c>
     </row>
     <row r="517" spans="1:10">
@@ -30438,7 +30438,7 @@
         <v>4951</v>
       </c>
       <c r="J521" t="s">
-        <v>4985</v>
+        <v>4986</v>
       </c>
     </row>
     <row r="522" spans="1:10">
@@ -30844,7 +30844,7 @@
         <v>4951</v>
       </c>
       <c r="J535" t="s">
-        <v>4985</v>
+        <v>4986</v>
       </c>
     </row>
     <row r="536" spans="1:10">
@@ -33512,7 +33512,7 @@
         <v>4951</v>
       </c>
       <c r="J627" t="s">
-        <v>4985</v>
+        <v>4986</v>
       </c>
     </row>
     <row r="628" spans="1:10">
@@ -34411,7 +34411,7 @@
         <v>4951</v>
       </c>
       <c r="J658" t="s">
-        <v>4985</v>
+        <v>4986</v>
       </c>
     </row>
     <row r="659" spans="1:10">
@@ -35281,7 +35281,7 @@
         <v>4951</v>
       </c>
       <c r="J688" t="s">
-        <v>4985</v>
+        <v>4986</v>
       </c>
     </row>
     <row r="689" spans="1:10">
@@ -35368,7 +35368,7 @@
         <v>4951</v>
       </c>
       <c r="J691" t="s">
-        <v>4985</v>
+        <v>4986</v>
       </c>
     </row>
     <row r="692" spans="1:10">
@@ -35861,7 +35861,7 @@
         <v>4951</v>
       </c>
       <c r="J708" t="s">
-        <v>4985</v>
+        <v>4986</v>
       </c>
     </row>
     <row r="709" spans="1:10">
@@ -36760,7 +36760,7 @@
         <v>4951</v>
       </c>
       <c r="J739" t="s">
-        <v>4985</v>
+        <v>4986</v>
       </c>
     </row>
     <row r="740" spans="1:10">
@@ -39107,7 +39107,7 @@
         <v>4974</v>
       </c>
       <c r="J816" t="s">
-        <v>4985</v>
+        <v>4986</v>
       </c>
     </row>
     <row r="817" spans="1:10">
@@ -40217,7 +40217,7 @@
         <v>4980</v>
       </c>
       <c r="J852" t="s">
-        <v>4985</v>
+        <v>4986</v>
       </c>
     </row>
     <row r="853" spans="1:10">
@@ -58626,7 +58626,7 @@
         <v>4974</v>
       </c>
       <c r="J1457" t="s">
-        <v>4985</v>
+        <v>4986</v>
       </c>
     </row>
     <row r="1458" spans="1:10">

</xml_diff>

<commit_message>
Update INARA 2026-09-22 09:41:45
</commit_message>
<xml_diff>
--- a/report_cleansing_ps.xlsx
+++ b/report_cleansing_ps.xlsx
@@ -24208,7 +24208,7 @@
         <v>6537</v>
       </c>
       <c r="J142" t="s">
-        <v>6571</v>
+        <v>6572</v>
       </c>
     </row>
     <row r="143" spans="1:10">
@@ -36066,7 +36066,7 @@
         <v>6537</v>
       </c>
       <c r="J551" t="s">
-        <v>6571</v>
+        <v>6572</v>
       </c>
     </row>
     <row r="552" spans="1:10">
@@ -50000,7 +50000,7 @@
         <v>6545</v>
       </c>
       <c r="J1029" t="s">
-        <v>6571</v>
+        <v>6572</v>
       </c>
     </row>
     <row r="1030" spans="1:10">
@@ -53959,7 +53959,7 @@
         <v>6545</v>
       </c>
       <c r="J1159" t="s">
-        <v>6571</v>
+        <v>6572</v>
       </c>
     </row>
     <row r="1160" spans="1:10">
@@ -55701,7 +55701,7 @@
         <v>6545</v>
       </c>
       <c r="J1217" t="s">
-        <v>6571</v>
+        <v>6572</v>
       </c>
     </row>
     <row r="1218" spans="1:10">
@@ -64282,7 +64282,7 @@
         <v>6566</v>
       </c>
       <c r="J1498" t="s">
-        <v>6571</v>
+        <v>6572</v>
       </c>
     </row>
     <row r="1499" spans="1:10">
@@ -67021,7 +67021,7 @@
         <v>6545</v>
       </c>
       <c r="J1588" t="s">
-        <v>6571</v>
+        <v>6572</v>
       </c>
     </row>
     <row r="1589" spans="1:10">
@@ -67108,7 +67108,7 @@
         <v>6545</v>
       </c>
       <c r="J1591" t="s">
-        <v>6571</v>
+        <v>6572</v>
       </c>
     </row>
     <row r="1592" spans="1:10">
@@ -74738,7 +74738,7 @@
         <v>6558</v>
       </c>
       <c r="J1842" t="s">
-        <v>6571</v>
+        <v>6572</v>
       </c>
     </row>
     <row r="1843" spans="1:10">
@@ -75789,7 +75789,7 @@
         <v>6545</v>
       </c>
       <c r="J1877" t="s">
-        <v>6571</v>
+        <v>6572</v>
       </c>
     </row>
     <row r="1878" spans="1:10">
@@ -87218,7 +87218,7 @@
         <v>6545</v>
       </c>
       <c r="J2250" t="s">
-        <v>6571</v>
+        <v>6572</v>
       </c>
     </row>
     <row r="2251" spans="1:10">

</xml_diff>

<commit_message>
Update INARA 2026-09-23 10:40:24
</commit_message>
<xml_diff>
--- a/report_cleansing_ps.xlsx
+++ b/report_cleansing_ps.xlsx
@@ -25114,7 +25114,7 @@
         <v>6896</v>
       </c>
       <c r="J136" t="s">
-        <v>6931</v>
+        <v>6932</v>
       </c>
     </row>
     <row r="137" spans="1:10">
@@ -26912,7 +26912,7 @@
         <v>6897</v>
       </c>
       <c r="J198" t="s">
-        <v>6931</v>
+        <v>6932</v>
       </c>
     </row>
     <row r="199" spans="1:10">
@@ -30044,7 +30044,7 @@
         <v>6897</v>
       </c>
       <c r="J306" t="s">
-        <v>6931</v>
+        <v>6932</v>
       </c>
     </row>
     <row r="307" spans="1:10">
@@ -30566,7 +30566,7 @@
         <v>6901</v>
       </c>
       <c r="J324" t="s">
-        <v>6931</v>
+        <v>6932</v>
       </c>
     </row>
     <row r="325" spans="1:10">
@@ -32045,7 +32045,7 @@
         <v>6897</v>
       </c>
       <c r="J375" t="s">
-        <v>6931</v>
+        <v>6932</v>
       </c>
     </row>
     <row r="376" spans="1:10">
@@ -40655,7 +40655,7 @@
         <v>6901</v>
       </c>
       <c r="J672" t="s">
-        <v>6931</v>
+        <v>6932</v>
       </c>
     </row>
     <row r="673" spans="1:10">
@@ -41032,7 +41032,7 @@
         <v>6897</v>
       </c>
       <c r="J685" t="s">
-        <v>6931</v>
+        <v>6932</v>
       </c>
     </row>
     <row r="686" spans="1:10">
@@ -41525,7 +41525,7 @@
         <v>6901</v>
       </c>
       <c r="J702" t="s">
-        <v>6931</v>
+        <v>6932</v>
       </c>
     </row>
     <row r="703" spans="1:10">
@@ -43410,7 +43410,7 @@
         <v>6896</v>
       </c>
       <c r="J767" t="s">
-        <v>6931</v>
+        <v>6932</v>
       </c>
     </row>
     <row r="768" spans="1:10">
@@ -46078,7 +46078,7 @@
         <v>6901</v>
       </c>
       <c r="J859" t="s">
-        <v>6931</v>
+        <v>6932</v>
       </c>
     </row>
     <row r="860" spans="1:10">
@@ -46513,7 +46513,7 @@
         <v>6901</v>
       </c>
       <c r="J874" t="s">
-        <v>6931</v>
+        <v>6932</v>
       </c>
     </row>
     <row r="875" spans="1:10">
@@ -48195,7 +48195,7 @@
         <v>6901</v>
       </c>
       <c r="J932" t="s">
-        <v>6931</v>
+        <v>6932</v>
       </c>
     </row>
     <row r="933" spans="1:10">
@@ -62106,7 +62106,7 @@
         <v>6922</v>
       </c>
       <c r="J1394" t="s">
-        <v>6931</v>
+        <v>6932</v>
       </c>
     </row>
     <row r="1395" spans="1:10">
@@ -74852,7 +74852,7 @@
         <v>6916</v>
       </c>
       <c r="J1812" t="s">
-        <v>6931</v>
+        <v>6932</v>
       </c>
     </row>
     <row r="1813" spans="1:10">
@@ -78636,7 +78636,7 @@
         <v>6908</v>
       </c>
       <c r="J1937" t="s">
-        <v>6931</v>
+        <v>6932</v>
       </c>
     </row>
     <row r="1938" spans="1:10">
@@ -90678,7 +90678,7 @@
         <v>6922</v>
       </c>
       <c r="J2330" t="s">
-        <v>6931</v>
+        <v>6932</v>
       </c>
     </row>
     <row r="2331" spans="1:10">
@@ -94963,7 +94963,7 @@
         <v>6908</v>
       </c>
       <c r="J2470" t="s">
-        <v>6931</v>
+        <v>6932</v>
       </c>
     </row>
     <row r="2471" spans="1:10">

</xml_diff>

<commit_message>
Update INARA 2026-09-25 10:00:37
</commit_message>
<xml_diff>
--- a/report_cleansing_ps.xlsx
+++ b/report_cleansing_ps.xlsx
@@ -52168,7 +52168,7 @@
         <v>7593</v>
       </c>
       <c r="J997" t="s">
-        <v>7627</v>
+        <v>7628</v>
       </c>
     </row>
     <row r="998" spans="1:10">
@@ -61605,7 +61605,7 @@
         <v>7618</v>
       </c>
       <c r="J1313" t="s">
-        <v>7627</v>
+        <v>7628</v>
       </c>
     </row>
     <row r="1314" spans="1:10">
@@ -64695,7 +64695,7 @@
         <v>7610</v>
       </c>
       <c r="J1415" t="s">
-        <v>7627</v>
+        <v>7628</v>
       </c>
     </row>
     <row r="1416" spans="1:10">
@@ -73424,7 +73424,7 @@
         <v>7610</v>
       </c>
       <c r="J1701" t="s">
-        <v>7627</v>
+        <v>7628</v>
       </c>
     </row>
     <row r="1702" spans="1:10">
@@ -76500,7 +76500,7 @@
         <v>7616</v>
       </c>
       <c r="J1802" t="s">
-        <v>7627</v>
+        <v>7628</v>
       </c>
     </row>
     <row r="1803" spans="1:10">

</xml_diff>